<commit_message>
delete old arb map
</commit_message>
<xml_diff>
--- a/docs/arb_stiffness.xlsx
+++ b/docs/arb_stiffness.xlsx
@@ -542,11 +542,11 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -632,19 +632,19 @@
     <xf numFmtId="0" fontId="13" fillId="11" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="18" fillId="15" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="18" fillId="15" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -662,7 +662,10 @@
     <xf numFmtId="176" fontId="17" fillId="14" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
@@ -672,9 +675,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1780,65 +1780,65 @@
     </row>
     <row r="4" spans="1:15" ht="26.1" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="1:15" ht="26.1" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="1" t="str">
+      <c r="B5" s="37" t="str">
         <f>IF(COUNT(Samples!H6:J17)=0,"待补节点坐标；暂无刚度结果。","")</f>
         <v/>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="26.1" customHeight="1">
@@ -2574,43 +2574,43 @@
     </row>
     <row r="49" spans="1:15" ht="26.1" customHeight="1">
       <c r="A49" s="1"/>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="G49" s="1" t="s">
+      <c r="G49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="H49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="I49" s="1" t="s">
+      <c r="I49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="J49" s="1" t="s">
+      <c r="J49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="K49" s="1" t="s">
+      <c r="K49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="L49" s="1" t="s">
+      <c r="L49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="M49" s="1" t="s">
+      <c r="M49" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="N49" s="1" t="s">
+      <c r="N49" s="37" t="s">
         <v>2</v>
       </c>
       <c r="O49" s="1"/>
@@ -2662,56 +2662,56 @@
     </row>
     <row r="2" spans="1:10" ht="27" customHeight="1">
       <c r="A2" s="15"/>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="27" customHeight="1">
       <c r="A3" s="15"/>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J3" s="15"/>
@@ -2721,25 +2721,25 @@
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="37" t="s">
+      <c r="G4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="37" t="s">
+      <c r="H4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="I4" s="38" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="15"/>
@@ -2915,56 +2915,56 @@
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1">
       <c r="A14" s="15"/>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="38" t="s">
+      <c r="C14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="38" t="s">
+      <c r="E14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="38" t="s">
+      <c r="F14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="38" t="s">
+      <c r="G14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="38" t="s">
+      <c r="H14" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="I14" s="38" t="s">
+      <c r="I14" s="39" t="s">
         <v>11</v>
       </c>
       <c r="J14" s="15"/>
     </row>
     <row r="15" spans="1:10" ht="27" customHeight="1">
       <c r="A15" s="15"/>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="39" t="s">
+      <c r="E15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="39" t="s">
+      <c r="G15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="39" t="s">
+      <c r="H15" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="39" t="s">
+      <c r="I15" s="40" t="s">
         <v>12</v>
       </c>
       <c r="J15" s="15"/>
@@ -3022,44 +3022,44 @@
     </row>
     <row r="20" spans="1:14" ht="27" customHeight="1">
       <c r="A20" s="15"/>
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="38" t="s">
+      <c r="D20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="38" t="s">
+      <c r="F20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="G20" s="38" t="s">
+      <c r="G20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="38" t="s">
+      <c r="H20" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="38" t="s">
+      <c r="I20" s="39" t="s">
         <v>18</v>
       </c>
       <c r="J20" s="15"/>
     </row>
     <row r="21" spans="1:14" ht="27" customHeight="1">
       <c r="A21" s="15"/>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="41"/>
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="1:14" ht="42" customHeight="1">
@@ -5485,13 +5485,13 @@
     </row>
     <row r="49" spans="1:13" ht="26.1" customHeight="1">
       <c r="A49" s="1"/>
-      <c r="B49" s="41" t="s">
+      <c r="B49" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C49" s="41" t="s">
+      <c r="C49" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D49" s="41" t="s">
+      <c r="D49" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E49" s="1"/>

</xml_diff>